<commit_message>
Release v1.0.0 final LUAD deployability audit package
</commit_message>
<xml_diff>
--- a/supplementary/Supplementary_Data_2A_reconstructed_282_exclusion_categories.xlsx
+++ b/supplementary/Supplementary_Data_2A_reconstructed_282_exclusion_categories.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manual_282_categories" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reconstructed_282_categories" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interpretation_notes" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
@@ -480,7 +480,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Author-provided manual table-screening aggregate category; no records assigned in the 282-count summary</t>
+          <t>Author-performed manual table-screening aggregate category; no records assigned in the 282-count summary</t>
         </is>
       </c>
       <c r="E2" s="2" t="n">
@@ -501,7 +501,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Author-provided manual table-screening aggregate category for the 282 pre-audit full-text-target exclusions</t>
+          <t>Author-performed manual table-screening aggregate category for the 282 pre-audit full-text-target exclusions</t>
         </is>
       </c>
       <c r="E3" s="2" t="n">
@@ -522,7 +522,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Author-provided manual table-screening aggregate category for the 282 pre-audit full-text-target exclusions</t>
+          <t>Author-performed manual table-screening aggregate category for the 282 pre-audit full-text-target exclusions</t>
         </is>
       </c>
       <c r="E4" s="2" t="n">
@@ -543,7 +543,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Author-provided manual table-screening aggregate category; no records assigned in the 282-count summary</t>
+          <t>Author-performed manual table-screening aggregate category; no records assigned in the 282-count summary</t>
         </is>
       </c>
       <c r="E5" s="2" t="n">
@@ -564,7 +564,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Author-provided manual table-screening aggregate category for the 282 pre-audit full-text-target exclusions</t>
+          <t>Author-performed manual table-screening aggregate category for the 282 pre-audit full-text-target exclusions</t>
         </is>
       </c>
       <c r="E6" s="2" t="n">
@@ -585,7 +585,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Author-provided manual table-screening aggregate category for the 282 pre-audit full-text-target exclusions</t>
+          <t>Author-performed manual table-screening aggregate category for the 282 pre-audit full-text-target exclusions</t>
         </is>
       </c>
       <c r="E7" s="2" t="n">
@@ -606,7 +606,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Author-provided manual table-screening aggregate category for the 282 pre-audit full-text-target exclusions</t>
+          <t>Author-performed manual table-screening aggregate category for the 282 pre-audit full-text-target exclusions</t>
         </is>
       </c>
       <c r="E8" s="2" t="n">
@@ -627,7 +627,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Author-provided manual table-screening aggregate category; no records assigned in the 282-count summary</t>
+          <t>Author-performed manual table-screening aggregate category; no records assigned in the 282-count summary</t>
         </is>
       </c>
       <c r="E9" s="2" t="n">
@@ -672,7 +672,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Aggregate author-provided manual table-screening reasons for 282 pre-audit full-text-target exclusions.</t>
+          <t>Aggregate author-performed manual table-screening reasons for 282 pre-audit full-text-target exclusions.</t>
         </is>
       </c>
     </row>
@@ -684,7 +684,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Do not treat as a verified 282-row PRISMA exclusion table.</t>
+          <t>Do not treat as a 282-row article-level bibliographic exclusion appendix.</t>
         </is>
       </c>
     </row>

</xml_diff>